<commit_message>
Further save of data
</commit_message>
<xml_diff>
--- a/Data/scenarios.xlsx
+++ b/Data/scenarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sandee\Documents\Github\STraM_ntnu_development\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26E5E6EF-4FC5-4EB3-B457-4DB170DAB952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DACD910D-FA66-4DBD-90FC-1BA5C01C2BB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-18120" yWindow="-7965" windowWidth="18240" windowHeight="28440" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3687" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3685" uniqueCount="63">
   <si>
     <t>Variability</t>
   </si>
@@ -17599,9 +17599,7 @@
       <c r="E1" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="F1" s="4"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
@@ -17621,9 +17619,7 @@
       <c r="E2" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>6</v>
-      </c>
+      <c r="F2" s="3"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3">

</xml_diff>

<commit_message>
Bug fix in scenario data
</commit_message>
<xml_diff>
--- a/Data/scenarios.xlsx
+++ b/Data/scenarios.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://studntnu-my.sharepoint.com/personal/steffejb_ntnu_no/Documents/Work/GitHub/STraM_ntnu_development/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sandee\Documents\Github\STraM_ntnu_development\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{5252CC3E-A50E-4DB5-8DFA-66AD561181FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E627CD8D-28A9-4B73-A7CF-91A9ACBBBFAE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C2130E0-FEB2-4346-BAE7-2BD990CEB925}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="28800" windowHeight="23400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-18120" yWindow="-7965" windowWidth="18240" windowHeight="28440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cost_factor" sheetId="10" r:id="rId1"/>
     <sheet name="demand_factor" sheetId="15" r:id="rId2"/>
     <sheet name="fuel_scenarios" sheetId="11" r:id="rId3"/>
-    <sheet name="fuel_scenarios_5" sheetId="14" r:id="rId4"/>
+    <sheet name="fuel_scenarios_16" sheetId="14" r:id="rId4"/>
     <sheet name="fuel_scenarios_demand" sheetId="13" r:id="rId5"/>
     <sheet name="fuel_scenario_det" sheetId="12" r:id="rId6"/>
     <sheet name="scenarios_base" sheetId="8" r:id="rId7"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3672" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3662" uniqueCount="71">
   <si>
     <t>Variability</t>
   </si>
@@ -603,7 +603,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C62B08C-45D2-4F7F-A1A1-F485128869A7}">
-  <dimension ref="A1:G824"/>
+  <dimension ref="A1:G826"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.28515625" bestFit="1" customWidth="1"/>
@@ -12723,19 +12723,19 @@
         <v>68</v>
       </c>
       <c r="B601">
-        <v>2023</v>
+        <v>2050</v>
       </c>
       <c r="C601" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D601" t="s">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="E601" t="s">
-        <v>55</v>
+        <v>11</v>
       </c>
       <c r="F601" s="3">
-        <v>0.9770072262166376</v>
+        <v>0.99047026671717431</v>
       </c>
       <c r="G601" s="3"/>
     </row>
@@ -12753,10 +12753,10 @@
         <v>8</v>
       </c>
       <c r="E602" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F602" s="3">
-        <v>0.96659211296828973</v>
+        <v>0.9770072262166376</v>
       </c>
       <c r="G602" s="3"/>
     </row>
@@ -12774,10 +12774,10 @@
         <v>8</v>
       </c>
       <c r="E603" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F603" s="3">
-        <v>0.98073208764779951</v>
+        <v>0.96659211296828973</v>
       </c>
       <c r="G603" s="3"/>
     </row>
@@ -12795,10 +12795,10 @@
         <v>8</v>
       </c>
       <c r="E604" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F604" s="3">
-        <v>0.9763680674587325</v>
+        <v>0.98073208764779951</v>
       </c>
       <c r="G604" s="3"/>
     </row>
@@ -12816,10 +12816,10 @@
         <v>8</v>
       </c>
       <c r="E605" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F605" s="3">
-        <v>0.98532183773215398</v>
+        <v>0.9763680674587325</v>
       </c>
       <c r="G605" s="3"/>
     </row>
@@ -12834,13 +12834,13 @@
         <v>19</v>
       </c>
       <c r="D606" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E606" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F606" s="3">
-        <v>0.97869656906053404</v>
+        <v>0.98532183773215398</v>
       </c>
       <c r="G606" s="3"/>
     </row>
@@ -12858,10 +12858,10 @@
         <v>13</v>
       </c>
       <c r="E607" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F607" s="3">
-        <v>0.96823287211849074</v>
+        <v>0.97869656906053404</v>
       </c>
       <c r="G607" s="3"/>
     </row>
@@ -12879,10 +12879,10 @@
         <v>13</v>
       </c>
       <c r="E608" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F608" s="3">
-        <v>0.98120477845085641</v>
+        <v>0.96823287211849074</v>
       </c>
       <c r="G608" s="3"/>
     </row>
@@ -12900,10 +12900,10 @@
         <v>13</v>
       </c>
       <c r="E609" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F609" s="3">
-        <v>0.97699617169756015</v>
+        <v>0.98120477845085641</v>
       </c>
       <c r="G609" s="3"/>
     </row>
@@ -12921,10 +12921,10 @@
         <v>13</v>
       </c>
       <c r="E610" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F610" s="3">
-        <v>0.98552323247933848</v>
+        <v>0.97699617169756015</v>
       </c>
       <c r="G610" s="3"/>
     </row>
@@ -12939,13 +12939,13 @@
         <v>19</v>
       </c>
       <c r="D611" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E611" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F611" s="3">
-        <v>0.9770007660165938</v>
+        <v>0.98552323247933848</v>
       </c>
       <c r="G611" s="3"/>
     </row>
@@ -12963,10 +12963,10 @@
         <v>14</v>
       </c>
       <c r="E612" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F612" s="3">
-        <v>0.96658599989356897</v>
+        <v>0.9770007660165938</v>
       </c>
       <c r="G612" s="3"/>
     </row>
@@ -12984,10 +12984,10 @@
         <v>14</v>
       </c>
       <c r="E613" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F613" s="3">
-        <v>0.98073002377074159</v>
+        <v>0.96658599989356897</v>
       </c>
       <c r="G613" s="3"/>
     </row>
@@ -13005,10 +13005,10 @@
         <v>14</v>
       </c>
       <c r="E614" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F614" s="3">
-        <v>0.97636541179631564</v>
+        <v>0.98073002377074159</v>
       </c>
       <c r="G614" s="3"/>
     </row>
@@ -13026,10 +13026,10 @@
         <v>14</v>
       </c>
       <c r="E615" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F615" s="3">
-        <v>0.98532105593669927</v>
+        <v>0.97636541179631564</v>
       </c>
       <c r="G615" s="3"/>
     </row>
@@ -13044,13 +13044,13 @@
         <v>19</v>
       </c>
       <c r="D616" t="s">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="E616" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F616" s="3">
-        <v>0.97698965288887907</v>
+        <v>0.98532105593669927</v>
       </c>
       <c r="G616" s="3"/>
     </row>
@@ -13068,10 +13068,10 @@
         <v>53</v>
       </c>
       <c r="E617" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F617" s="3">
-        <v>0.96657548670816806</v>
+        <v>0.97698965288887907</v>
       </c>
       <c r="G617" s="3"/>
     </row>
@@ -13089,10 +13089,10 @@
         <v>53</v>
       </c>
       <c r="E618" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F618" s="3">
-        <v>0.98072744153701752</v>
+        <v>0.96657548670816806</v>
       </c>
       <c r="G618" s="3"/>
     </row>
@@ -13110,10 +13110,10 @@
         <v>53</v>
       </c>
       <c r="E619" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F619" s="3">
-        <v>0.97636187464048774</v>
+        <v>0.98072744153701752</v>
       </c>
       <c r="G619" s="3"/>
     </row>
@@ -13131,10 +13131,10 @@
         <v>53</v>
       </c>
       <c r="E620" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F620" s="3">
-        <v>0.98531987448985237</v>
+        <v>0.97636187464048774</v>
       </c>
       <c r="G620" s="3"/>
     </row>
@@ -13143,19 +13143,19 @@
         <v>68</v>
       </c>
       <c r="B621">
-        <v>2034</v>
+        <v>2023</v>
       </c>
       <c r="C621" t="s">
         <v>19</v>
       </c>
       <c r="D621" t="s">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="E621" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F621" s="3">
-        <v>0.91435117400938704</v>
+        <v>0.98531987448985237</v>
       </c>
       <c r="G621" s="3"/>
     </row>
@@ -13173,10 +13173,10 @@
         <v>8</v>
       </c>
       <c r="E622" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F622" s="3">
-        <v>0.86917560791901605</v>
+        <v>0.91435117400938704</v>
       </c>
       <c r="G622" s="3"/>
     </row>
@@ -13194,10 +13194,10 @@
         <v>8</v>
       </c>
       <c r="E623" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F623" s="3">
-        <v>0.96876832520440281</v>
+        <v>0.86917560791901605</v>
       </c>
       <c r="G623" s="3"/>
     </row>
@@ -13215,10 +13215,10 @@
         <v>8</v>
       </c>
       <c r="E624" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F624" s="3">
-        <v>0.96402435867415437</v>
+        <v>0.96876832520440281</v>
       </c>
       <c r="G624" s="3"/>
     </row>
@@ -13236,10 +13236,10 @@
         <v>8</v>
       </c>
       <c r="E625" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F625" s="3">
-        <v>0.96958260356281867</v>
+        <v>0.96402435867415437</v>
       </c>
       <c r="G625" s="3"/>
     </row>
@@ -13254,13 +13254,13 @@
         <v>19</v>
       </c>
       <c r="D626" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E626" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F626" s="3">
-        <v>0.92125344647449081</v>
+        <v>0.96958260356281867</v>
       </c>
       <c r="G626" s="3"/>
     </row>
@@ -13278,10 +13278,10 @@
         <v>13</v>
       </c>
       <c r="E627" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F627" s="3">
-        <v>0.87658265414421443</v>
+        <v>0.92125344647449081</v>
       </c>
       <c r="G627" s="3"/>
     </row>
@@ -13299,10 +13299,10 @@
         <v>13</v>
       </c>
       <c r="E628" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F628" s="3">
-        <v>0.96964336574193677</v>
+        <v>0.87658265414421443</v>
       </c>
       <c r="G628" s="3"/>
     </row>
@@ -13320,10 +13320,10 @@
         <v>13</v>
       </c>
       <c r="E629" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F629" s="3">
-        <v>0.96505160615423602</v>
+        <v>0.96964336574193677</v>
       </c>
       <c r="G629" s="3"/>
     </row>
@@ -13341,10 +13341,10 @@
         <v>13</v>
       </c>
       <c r="E630" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F630" s="3">
-        <v>0.97018743860908951</v>
+        <v>0.96505160615423602</v>
       </c>
       <c r="G630" s="3"/>
     </row>
@@ -13359,13 +13359,13 @@
         <v>19</v>
       </c>
       <c r="D631" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E631" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F631" s="3">
-        <v>0.91432457403815048</v>
+        <v>0.97018743860908951</v>
       </c>
       <c r="G631" s="3"/>
     </row>
@@ -13383,10 +13383,10 @@
         <v>14</v>
       </c>
       <c r="E632" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F632" s="3">
-        <v>0.86914779066455838</v>
+        <v>0.91432457403815048</v>
       </c>
       <c r="G632" s="3"/>
     </row>
@@ -13404,10 +13404,10 @@
         <v>14</v>
       </c>
       <c r="E633" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F633" s="3">
-        <v>0.96876450432493588</v>
+        <v>0.86914779066455838</v>
       </c>
       <c r="G633" s="3"/>
     </row>
@@ -13425,10 +13425,10 @@
         <v>14</v>
       </c>
       <c r="E634" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F634" s="3">
-        <v>0.96402001447221397</v>
+        <v>0.96876450432493588</v>
       </c>
       <c r="G634" s="3"/>
     </row>
@@ -13446,10 +13446,10 @@
         <v>14</v>
       </c>
       <c r="E635" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F635" s="3">
-        <v>0.96958024082672667</v>
+        <v>0.96402001447221397</v>
       </c>
       <c r="G635" s="3"/>
     </row>
@@ -13464,13 +13464,13 @@
         <v>19</v>
       </c>
       <c r="D636" t="s">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="E636" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F636" s="3">
-        <v>0.91427881188292126</v>
+        <v>0.96958024082672667</v>
       </c>
       <c r="G636" s="3"/>
     </row>
@@ -13488,10 +13488,10 @@
         <v>53</v>
       </c>
       <c r="E637" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F637" s="3">
-        <v>0.86909994705962601</v>
+        <v>0.91427881188292126</v>
       </c>
       <c r="G637" s="3"/>
     </row>
@@ -13509,10 +13509,10 @@
         <v>53</v>
       </c>
       <c r="E638" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F638" s="3">
-        <v>0.96875969233905002</v>
+        <v>0.86909994705962601</v>
       </c>
       <c r="G638" s="3"/>
     </row>
@@ -13530,10 +13530,10 @@
         <v>53</v>
       </c>
       <c r="E639" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F639" s="3">
-        <v>0.96401420917704694</v>
+        <v>0.96875969233905002</v>
       </c>
       <c r="G639" s="3"/>
     </row>
@@ -13551,10 +13551,10 @@
         <v>53</v>
       </c>
       <c r="E640" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F640" s="3">
-        <v>0.96957667004842407</v>
+        <v>0.96401420917704694</v>
       </c>
       <c r="G640" s="3"/>
     </row>
@@ -13563,19 +13563,19 @@
         <v>68</v>
       </c>
       <c r="B641">
-        <v>2050</v>
+        <v>2034</v>
       </c>
       <c r="C641" t="s">
         <v>19</v>
       </c>
       <c r="D641" t="s">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="E641" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F641" s="3">
-        <v>0.90766002054982542</v>
+        <v>0.96957667004842407</v>
       </c>
       <c r="G641" s="3"/>
     </row>
@@ -13593,10 +13593,10 @@
         <v>8</v>
       </c>
       <c r="E642" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F642" s="3">
-        <v>0.85176875751396475</v>
+        <v>0.90766002054982542</v>
       </c>
       <c r="G642" s="3"/>
     </row>
@@ -13614,10 +13614,10 @@
         <v>8</v>
       </c>
       <c r="E643" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F643" s="3">
-        <v>0.95215044477953137</v>
+        <v>0.85176875751396475</v>
       </c>
       <c r="G643" s="3"/>
     </row>
@@ -13635,10 +13635,10 @@
         <v>8</v>
       </c>
       <c r="E644" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F644" s="3">
-        <v>0.94685336831016231</v>
+        <v>0.95215044477953137</v>
       </c>
       <c r="G644" s="3"/>
     </row>
@@ -13656,10 +13656,10 @@
         <v>8</v>
       </c>
       <c r="E645" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F645" s="3">
-        <v>0.94776591748146899</v>
+        <v>0.94685336831016231</v>
       </c>
       <c r="G645" s="3"/>
     </row>
@@ -13674,13 +13674,13 @@
         <v>19</v>
       </c>
       <c r="D646" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E646" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F646" s="3">
-        <v>0.91559876013359376</v>
+        <v>0.94776591748146899</v>
       </c>
       <c r="G646" s="3"/>
     </row>
@@ -13698,10 +13698,10 @@
         <v>13</v>
       </c>
       <c r="E647" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F647" s="3">
-        <v>0.86116577921306381</v>
+        <v>0.91559876013359376</v>
       </c>
       <c r="G647" s="3"/>
     </row>
@@ -13719,10 +13719,10 @@
         <v>13</v>
       </c>
       <c r="E648" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F648" s="3">
-        <v>0.9541155842108211</v>
+        <v>0.86116577921306381</v>
       </c>
       <c r="G648" s="3"/>
     </row>
@@ -13740,10 +13740,10 @@
         <v>13</v>
       </c>
       <c r="E649" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F649" s="3">
-        <v>0.949001835494931</v>
+        <v>0.9541155842108211</v>
       </c>
       <c r="G649" s="3"/>
     </row>
@@ -13761,10 +13761,10 @@
         <v>13</v>
       </c>
       <c r="E650" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F650" s="3">
-        <v>0.94940128664286627</v>
+        <v>0.949001835494931</v>
       </c>
       <c r="G650" s="3"/>
     </row>
@@ -13779,13 +13779,13 @@
         <v>19</v>
       </c>
       <c r="D651" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E651" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F651" s="3">
-        <v>0.90762924530104505</v>
+        <v>0.94940128664286627</v>
       </c>
       <c r="G651" s="3"/>
     </row>
@@ -13803,10 +13803,10 @@
         <v>14</v>
       </c>
       <c r="E652" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F652" s="3">
-        <v>0.85173321059722651</v>
+        <v>0.90762924530104505</v>
       </c>
       <c r="G652" s="3"/>
     </row>
@@ -13824,10 +13824,10 @@
         <v>14</v>
       </c>
       <c r="E653" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F653" s="3">
-        <v>0.95214200486725753</v>
+        <v>0.85173321059722651</v>
       </c>
       <c r="G653" s="3"/>
     </row>
@@ -13845,10 +13845,10 @@
         <v>14</v>
       </c>
       <c r="E654" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F654" s="3">
-        <v>0.94684431062079577</v>
+        <v>0.95214200486725753</v>
       </c>
       <c r="G654" s="3"/>
     </row>
@@ -13866,10 +13866,10 @@
         <v>14</v>
       </c>
       <c r="E655" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F655" s="3">
-        <v>0.94775945341476442</v>
+        <v>0.94684431062079577</v>
       </c>
       <c r="G655" s="3"/>
     </row>
@@ -13884,13 +13884,13 @@
         <v>19</v>
       </c>
       <c r="D656" t="s">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="E656" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F656" s="3">
-        <v>0.90757629679633478</v>
+        <v>0.94775945341476442</v>
       </c>
       <c r="G656" s="3"/>
     </row>
@@ -13908,10 +13908,10 @@
         <v>53</v>
       </c>
       <c r="E657" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F657" s="3">
-        <v>0.85167206803064044</v>
+        <v>0.90757629679633478</v>
       </c>
       <c r="G657" s="3"/>
     </row>
@@ -13929,10 +13929,10 @@
         <v>53</v>
       </c>
       <c r="E658" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F658" s="3">
-        <v>0.95213077402582114</v>
+        <v>0.85167206803064044</v>
       </c>
       <c r="G658" s="3"/>
     </row>
@@ -13950,10 +13950,10 @@
         <v>53</v>
       </c>
       <c r="E659" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F659" s="3">
-        <v>0.94683186653150608</v>
+        <v>0.95213077402582114</v>
       </c>
       <c r="G659" s="3"/>
     </row>
@@ -13971,37 +13971,37 @@
         <v>53</v>
       </c>
       <c r="E660" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F660" s="3">
-        <v>0.94774968320813291</v>
+        <v>0.94683186653150608</v>
       </c>
       <c r="G660" s="3"/>
     </row>
     <row r="661" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A661" t="s">
-        <v>16</v>
+        <v>68</v>
       </c>
       <c r="B661">
-        <v>2023</v>
+        <v>2050</v>
       </c>
       <c r="C661" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="D661" t="s">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="E661" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F661" s="3">
-        <v>1.0015069351213199</v>
+        <v>0.94774968320813291</v>
       </c>
       <c r="G661" s="3"/>
     </row>
     <row r="662" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A662" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B662">
         <v>2023</v>
@@ -14013,16 +14013,16 @@
         <v>8</v>
       </c>
       <c r="E662" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F662" s="3">
-        <v>1.0034853252281759</v>
+        <v>1.0015069351213199</v>
       </c>
       <c r="G662" s="3"/>
     </row>
     <row r="663" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A663" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B663">
         <v>2023</v>
@@ -14034,16 +14034,16 @@
         <v>8</v>
       </c>
       <c r="E663" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F663" s="3">
-        <v>1.007671648431463</v>
+        <v>1.0034853252281759</v>
       </c>
       <c r="G663" s="3"/>
     </row>
     <row r="664" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A664" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B664">
         <v>2023</v>
@@ -14052,19 +14052,19 @@
         <v>7</v>
       </c>
       <c r="D664" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E664" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F664" s="3">
-        <v>1.0026204117499469</v>
+        <v>1.007671648431463</v>
       </c>
       <c r="G664" s="3"/>
     </row>
     <row r="665" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A665" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B665">
         <v>2023</v>
@@ -14076,16 +14076,16 @@
         <v>12</v>
       </c>
       <c r="E665" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F665" s="3">
-        <v>1.0063539041135863</v>
+        <v>1.0026204117499469</v>
       </c>
       <c r="G665" s="3"/>
     </row>
     <row r="666" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A666" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B666">
         <v>2023</v>
@@ -14097,16 +14097,16 @@
         <v>12</v>
       </c>
       <c r="E666" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F666" s="3">
-        <v>1.0130223752431446</v>
+        <v>1.0063539041135863</v>
       </c>
       <c r="G666" s="3"/>
     </row>
     <row r="667" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A667" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B667">
         <v>2023</v>
@@ -14115,19 +14115,19 @@
         <v>7</v>
       </c>
       <c r="D667" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E667" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F667" s="3">
-        <v>1.0025961210196472</v>
+        <v>1.0130223752431446</v>
       </c>
       <c r="G667" s="3"/>
     </row>
     <row r="668" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A668" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B668">
         <v>2023</v>
@@ -14139,16 +14139,16 @@
         <v>13</v>
       </c>
       <c r="E668" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F668" s="3">
-        <v>1.006247322328474</v>
+        <v>1.0025961210196472</v>
       </c>
       <c r="G668" s="3"/>
     </row>
     <row r="669" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A669" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B669">
         <v>2023</v>
@@ -14160,16 +14160,16 @@
         <v>13</v>
       </c>
       <c r="E669" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F669" s="3">
-        <v>1.0128183840745999</v>
+        <v>1.006247322328474</v>
       </c>
       <c r="G669" s="3"/>
     </row>
     <row r="670" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A670" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B670">
         <v>2023</v>
@@ -14178,19 +14178,19 @@
         <v>7</v>
       </c>
       <c r="D670" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E670" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F670" s="3">
-        <v>1.0020278899208586</v>
+        <v>1.0128183840745999</v>
       </c>
       <c r="G670" s="3"/>
     </row>
     <row r="671" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A671" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B671">
         <v>2023</v>
@@ -14202,16 +14202,16 @@
         <v>14</v>
       </c>
       <c r="E671" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F671" s="3">
-        <v>1.0047833101675256</v>
+        <v>1.0020278899208586</v>
       </c>
       <c r="G671" s="3"/>
     </row>
     <row r="672" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A672" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B672">
         <v>2023</v>
@@ -14223,16 +14223,16 @@
         <v>14</v>
       </c>
       <c r="E672" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F672" s="3">
-        <v>1.0101830043975053</v>
+        <v>1.0047833101675256</v>
       </c>
       <c r="G672" s="3"/>
     </row>
     <row r="673" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A673" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B673">
         <v>2023</v>
@@ -14241,19 +14241,19 @@
         <v>7</v>
       </c>
       <c r="D673" t="s">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="E673" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F673" s="3">
-        <v>1.0022898019193085</v>
+        <v>1.0101830043975053</v>
       </c>
       <c r="G673" s="3"/>
     </row>
     <row r="674" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A674" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B674">
         <v>2023</v>
@@ -14265,16 +14265,16 @@
         <v>53</v>
       </c>
       <c r="E674" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F674" s="3">
-        <v>1.0054492060826372</v>
+        <v>1.0022898019193085</v>
       </c>
       <c r="G674" s="3"/>
     </row>
     <row r="675" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A675" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B675">
         <v>2023</v>
@@ -14286,37 +14286,37 @@
         <v>53</v>
       </c>
       <c r="E675" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F675" s="3">
-        <v>1.0114055060280722</v>
+        <v>1.0054492060826372</v>
       </c>
       <c r="G675" s="3"/>
     </row>
     <row r="676" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A676" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B676">
-        <v>2034</v>
+        <v>2023</v>
       </c>
       <c r="C676" t="s">
         <v>7</v>
       </c>
       <c r="D676" t="s">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="E676" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F676" s="3">
-        <v>1.0057381105465133</v>
+        <v>1.0114055060280722</v>
       </c>
       <c r="G676" s="3"/>
     </row>
     <row r="677" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A677" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B677">
         <v>2034</v>
@@ -14328,16 +14328,16 @@
         <v>8</v>
       </c>
       <c r="E677" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F677" s="3">
-        <v>1</v>
+        <v>1.0057381105465133</v>
       </c>
       <c r="G677" s="3"/>
     </row>
     <row r="678" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A678" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B678">
         <v>2034</v>
@@ -14349,16 +14349,16 @@
         <v>8</v>
       </c>
       <c r="E678" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F678" s="3">
-        <v>1.0068802632607898</v>
+        <v>1</v>
       </c>
       <c r="G678" s="3"/>
     </row>
     <row r="679" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A679" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B679">
         <v>2034</v>
@@ -14367,19 +14367,19 @@
         <v>7</v>
       </c>
       <c r="D679" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E679" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F679" s="3">
-        <v>1.0101646491172152</v>
+        <v>1.0068802632607898</v>
       </c>
       <c r="G679" s="3"/>
     </row>
     <row r="680" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A680" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B680">
         <v>2034</v>
@@ -14391,16 +14391,16 @@
         <v>12</v>
       </c>
       <c r="E680" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F680" s="3">
-        <v>1.0058089145035107</v>
+        <v>1.0101646491172152</v>
       </c>
       <c r="G680" s="3"/>
     </row>
     <row r="681" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A681" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B681">
         <v>2034</v>
@@ -14412,16 +14412,16 @@
         <v>12</v>
       </c>
       <c r="E681" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F681" s="3">
-        <v>1.0117644433302788</v>
+        <v>1.0058089145035107</v>
       </c>
       <c r="G681" s="3"/>
     </row>
     <row r="682" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A682" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B682">
         <v>2034</v>
@@ -14430,19 +14430,19 @@
         <v>7</v>
       </c>
       <c r="D682" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E682" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F682" s="3">
-        <v>1.0100630394500727</v>
+        <v>1.0117644433302788</v>
       </c>
       <c r="G682" s="3"/>
     </row>
     <row r="683" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A683" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B683">
         <v>2034</v>
@@ -14454,16 +14454,16 @@
         <v>13</v>
       </c>
       <c r="E683" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F683" s="3">
-        <v>1.0057429832570657</v>
+        <v>1.0100630394500727</v>
       </c>
       <c r="G683" s="3"/>
     </row>
     <row r="684" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A684" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B684">
         <v>2034</v>
@@ -14475,16 +14475,16 @@
         <v>13</v>
       </c>
       <c r="E684" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F684" s="3">
-        <v>1.0116239854743765</v>
+        <v>1.0057429832570657</v>
       </c>
       <c r="G684" s="3"/>
     </row>
     <row r="685" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A685" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B685">
         <v>2034</v>
@@ -14493,19 +14493,19 @@
         <v>7</v>
       </c>
       <c r="D685" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E685" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F685" s="3">
-        <v>1.0077878819602768</v>
+        <v>1.0116239854743765</v>
       </c>
       <c r="G685" s="3"/>
     </row>
     <row r="686" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A686" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B686">
         <v>2034</v>
@@ -14517,16 +14517,16 @@
         <v>14</v>
       </c>
       <c r="E686" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F686" s="3">
-        <v>1.0044149811878662</v>
+        <v>1.0077878819602768</v>
       </c>
       <c r="G686" s="3"/>
     </row>
     <row r="687" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A687" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B687">
         <v>2034</v>
@@ -14538,16 +14538,16 @@
         <v>14</v>
       </c>
       <c r="E687" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F687" s="3">
-        <v>1.0091762699604205</v>
+        <v>1.0044149811878662</v>
       </c>
       <c r="G687" s="3"/>
     </row>
     <row r="688" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A688" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B688">
         <v>2034</v>
@@ -14556,19 +14556,19 @@
         <v>7</v>
       </c>
       <c r="D688" t="s">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="E688" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F688" s="3">
-        <v>1.0088312098768086</v>
+        <v>1.0091762699604205</v>
       </c>
       <c r="G688" s="3"/>
     </row>
     <row r="689" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A689" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B689">
         <v>2034</v>
@@ -14580,16 +14580,16 @@
         <v>53</v>
       </c>
       <c r="E689" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F689" s="3">
-        <v>1.0050212900291551</v>
+        <v>1.0088312098768086</v>
       </c>
       <c r="G689" s="3"/>
     </row>
     <row r="690" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A690" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B690">
         <v>2034</v>
@@ -14601,37 +14601,37 @@
         <v>53</v>
       </c>
       <c r="E690" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F690" s="3">
-        <v>1.0103095053014599</v>
+        <v>1.0050212900291551</v>
       </c>
       <c r="G690" s="3"/>
     </row>
     <row r="691" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A691" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B691">
-        <v>2050</v>
+        <v>2034</v>
       </c>
       <c r="C691" t="s">
         <v>7</v>
       </c>
       <c r="D691" t="s">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="E691" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F691" s="3">
-        <v>1.0088327504773722</v>
+        <v>1.0103095053014599</v>
       </c>
       <c r="G691" s="3"/>
     </row>
     <row r="692" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A692" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B692">
         <v>2050</v>
@@ -14643,16 +14643,16 @@
         <v>8</v>
       </c>
       <c r="E692" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F692" s="3">
-        <v>1</v>
+        <v>1.0088327504773722</v>
       </c>
       <c r="G692" s="3"/>
     </row>
     <row r="693" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A693" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B693">
         <v>2050</v>
@@ -14664,16 +14664,16 @@
         <v>8</v>
       </c>
       <c r="E693" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F693" s="3">
-        <v>1.0053120928101715</v>
+        <v>1</v>
       </c>
       <c r="G693" s="3"/>
     </row>
     <row r="694" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A694" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B694">
         <v>2050</v>
@@ -14682,19 +14682,19 @@
         <v>7</v>
       </c>
       <c r="D694" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E694" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F694" s="3">
-        <v>1.0158547406177889</v>
+        <v>1.0053120928101715</v>
       </c>
       <c r="G694" s="3"/>
     </row>
     <row r="695" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A695" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B695">
         <v>2050</v>
@@ -14706,16 +14706,16 @@
         <v>12</v>
       </c>
       <c r="E695" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F695" s="3">
-        <v>1.0047848691101033</v>
+        <v>1.0158547406177889</v>
       </c>
       <c r="G695" s="3"/>
     </row>
     <row r="696" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A696" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B696">
         <v>2050</v>
@@ -14727,16 +14727,16 @@
         <v>12</v>
       </c>
       <c r="E696" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F696" s="3">
-        <v>1.0092753157463279</v>
+        <v>1.0047848691101033</v>
       </c>
       <c r="G696" s="3"/>
     </row>
     <row r="697" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A697" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B697">
         <v>2050</v>
@@ -14745,19 +14745,19 @@
         <v>7</v>
       </c>
       <c r="D697" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E697" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F697" s="3">
-        <v>1.0156847642829907</v>
+        <v>1.0092753157463279</v>
       </c>
       <c r="G697" s="3"/>
     </row>
     <row r="698" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A698" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B698">
         <v>2050</v>
@@ -14769,16 +14769,16 @@
         <v>13</v>
       </c>
       <c r="E698" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F698" s="3">
-        <v>1.0047388122631626</v>
+        <v>1.0156847642829907</v>
       </c>
       <c r="G698" s="3"/>
     </row>
     <row r="699" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A699" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B699">
         <v>2050</v>
@@ -14790,16 +14790,16 @@
         <v>13</v>
       </c>
       <c r="E699" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F699" s="3">
-        <v>1.0091808848640174</v>
+        <v>1.0047388122631626</v>
       </c>
       <c r="G699" s="3"/>
     </row>
     <row r="700" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A700" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B700">
         <v>2050</v>
@@ -14808,19 +14808,19 @@
         <v>7</v>
       </c>
       <c r="D700" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E700" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F700" s="3">
-        <v>1.0120596421280725</v>
+        <v>1.0091808848640174</v>
       </c>
       <c r="G700" s="3"/>
     </row>
     <row r="701" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A701" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B701">
         <v>2050</v>
@@ -14832,16 +14832,16 @@
         <v>14</v>
       </c>
       <c r="E701" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F701" s="3">
-        <v>1.0036375261764166</v>
+        <v>1.0120596421280725</v>
       </c>
       <c r="G701" s="3"/>
     </row>
     <row r="702" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A702" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B702">
         <v>2050</v>
@@ -14853,16 +14853,16 @@
         <v>14</v>
       </c>
       <c r="E702" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F702" s="3">
-        <v>1.0071602167883063</v>
+        <v>1.0036375261764166</v>
       </c>
       <c r="G702" s="3"/>
     </row>
     <row r="703" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A703" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B703">
         <v>2050</v>
@@ -14871,19 +14871,19 @@
         <v>7</v>
       </c>
       <c r="D703" t="s">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="E703" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F703" s="3">
-        <v>1.0137159413503023</v>
+        <v>1.0071602167883063</v>
       </c>
       <c r="G703" s="3"/>
     </row>
     <row r="704" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A704" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B704">
         <v>2050</v>
@@ -14895,16 +14895,16 @@
         <v>53</v>
       </c>
       <c r="E704" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F704" s="3">
-        <v>1.0041402580933472</v>
+        <v>1.0137159413503023</v>
       </c>
       <c r="G704" s="3"/>
     </row>
     <row r="705" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A705" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B705">
         <v>2050</v>
@@ -14916,37 +14916,37 @@
         <v>53</v>
       </c>
       <c r="E705" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F705" s="3">
-        <v>1.0080904455741324</v>
+        <v>1.0041402580933472</v>
       </c>
       <c r="G705" s="3"/>
     </row>
     <row r="706" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A706" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B706">
-        <v>2023</v>
+        <v>2050</v>
       </c>
       <c r="C706" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="D706" t="s">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="E706" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F706" s="3">
-        <v>1.0041931965042568</v>
+        <v>1.0080904455741324</v>
       </c>
       <c r="G706" s="3"/>
     </row>
     <row r="707" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A707" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B707">
         <v>2023</v>
@@ -14958,16 +14958,16 @@
         <v>8</v>
       </c>
       <c r="E707" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F707" s="3">
-        <v>1.0118750052493906</v>
+        <v>1.0041931965042568</v>
       </c>
       <c r="G707" s="3"/>
     </row>
     <row r="708" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A708" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B708">
         <v>2023</v>
@@ -14979,16 +14979,16 @@
         <v>8</v>
       </c>
       <c r="E708" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F708" s="3">
-        <v>1.0092790346711054</v>
+        <v>1.0118750052493906</v>
       </c>
       <c r="G708" s="3"/>
     </row>
     <row r="709" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A709" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B709">
         <v>2023</v>
@@ -15000,16 +15000,16 @@
         <v>8</v>
       </c>
       <c r="E709" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F709" s="3">
-        <v>1.0164893257649426</v>
+        <v>1.0092790346711054</v>
       </c>
       <c r="G709" s="3"/>
     </row>
     <row r="710" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A710" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B710">
         <v>2023</v>
@@ -15018,19 +15018,19 @@
         <v>17</v>
       </c>
       <c r="D710" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E710" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F710" s="3">
-        <v>1.0041618763004256</v>
+        <v>1.0164893257649426</v>
       </c>
       <c r="G710" s="3"/>
     </row>
     <row r="711" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A711" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B711">
         <v>2023</v>
@@ -15042,16 +15042,16 @@
         <v>12</v>
       </c>
       <c r="E711" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F711" s="3">
-        <v>1.0117660742537415</v>
+        <v>1.0041618763004256</v>
       </c>
       <c r="G711" s="3"/>
     </row>
     <row r="712" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A712" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B712">
         <v>2023</v>
@@ -15063,16 +15063,16 @@
         <v>12</v>
       </c>
       <c r="E712" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F712" s="3">
-        <v>1.0092166737222432</v>
+        <v>1.0117660742537415</v>
       </c>
       <c r="G712" s="3"/>
     </row>
     <row r="713" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A713" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B713">
         <v>2023</v>
@@ -15084,16 +15084,16 @@
         <v>12</v>
       </c>
       <c r="E713" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F713" s="3">
-        <v>1.0164015885776378</v>
+        <v>1.0092166737222432</v>
       </c>
       <c r="G713" s="3"/>
     </row>
     <row r="714" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A714" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B714">
         <v>2023</v>
@@ -15102,19 +15102,19 @@
         <v>17</v>
       </c>
       <c r="D714" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E714" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F714" s="3">
-        <v>1.0044060679171694</v>
+        <v>1.0164015885776378</v>
       </c>
       <c r="G714" s="3"/>
     </row>
     <row r="715" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A715" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B715">
         <v>2023</v>
@@ -15126,16 +15126,16 @@
         <v>13</v>
       </c>
       <c r="E715" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F715" s="3">
-        <v>1.0126254110059707</v>
+        <v>1.0044060679171694</v>
       </c>
       <c r="G715" s="3"/>
     </row>
     <row r="716" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A716" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B716">
         <v>2023</v>
@@ -15147,16 +15147,16 @@
         <v>13</v>
       </c>
       <c r="E716" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F716" s="3">
-        <v>1.0097039213633152</v>
+        <v>1.0126254110059707</v>
       </c>
       <c r="G716" s="3"/>
     </row>
     <row r="717" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A717" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B717">
         <v>2023</v>
@@ -15168,16 +15168,16 @@
         <v>13</v>
       </c>
       <c r="E717" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F717" s="3">
-        <v>1.0170781763400143</v>
+        <v>1.0097039213633152</v>
       </c>
       <c r="G717" s="3"/>
     </row>
     <row r="718" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A718" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B718">
         <v>2023</v>
@@ -15186,19 +15186,19 @@
         <v>17</v>
       </c>
       <c r="D718" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E718" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F718" s="3">
-        <v>1.0029097819035671</v>
+        <v>1.0170781763400143</v>
       </c>
       <c r="G718" s="3"/>
     </row>
     <row r="719" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A719" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B719">
         <v>2023</v>
@@ -15210,16 +15210,16 @@
         <v>14</v>
       </c>
       <c r="E719" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F719" s="3">
-        <v>1.0076979756882698</v>
+        <v>1.0029097819035671</v>
       </c>
       <c r="G719" s="3"/>
     </row>
     <row r="720" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A720" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B720">
         <v>2023</v>
@@ -15231,16 +15231,16 @@
         <v>14</v>
       </c>
       <c r="E720" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F720" s="3">
-        <v>1.0066322349980039</v>
+        <v>1.0076979756882698</v>
       </c>
       <c r="G720" s="3"/>
     </row>
     <row r="721" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A721" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B721">
         <v>2023</v>
@@ -15252,16 +15252,16 @@
         <v>14</v>
       </c>
       <c r="E721" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F721" s="3">
-        <v>1.0125439730453332</v>
+        <v>1.0066322349980039</v>
       </c>
       <c r="G721" s="3"/>
     </row>
     <row r="722" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A722" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B722">
         <v>2023</v>
@@ -15270,19 +15270,19 @@
         <v>17</v>
       </c>
       <c r="D722" t="s">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="E722" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F722" s="3">
-        <v>1.0042400707597854</v>
+        <v>1.0125439730453332</v>
       </c>
       <c r="G722" s="3"/>
     </row>
     <row r="723" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A723" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B723">
         <v>2023</v>
@@ -15294,16 +15294,16 @@
         <v>53</v>
       </c>
       <c r="E723" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F723" s="3">
-        <v>1.0120387346215614</v>
+        <v>1.0042400707597854</v>
       </c>
       <c r="G723" s="3"/>
     </row>
     <row r="724" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A724" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B724">
         <v>2023</v>
@@ -15315,16 +15315,16 @@
         <v>53</v>
       </c>
       <c r="E724" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F724" s="3">
-        <v>1.0093735899742056</v>
+        <v>1.0120387346215614</v>
       </c>
       <c r="G724" s="3"/>
     </row>
     <row r="725" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A725" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B725">
         <v>2023</v>
@@ -15336,37 +15336,37 @@
         <v>53</v>
       </c>
       <c r="E725" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F725" s="3">
-        <v>1.0166209081526265</v>
+        <v>1.0093735899742056</v>
       </c>
       <c r="G725" s="3"/>
     </row>
     <row r="726" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A726" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B726">
-        <v>2034</v>
+        <v>2023</v>
       </c>
       <c r="C726" t="s">
         <v>17</v>
       </c>
       <c r="D726" t="s">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="E726" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F726" s="3">
-        <v>1.0178559493587218</v>
+        <v>1.0166209081526265</v>
       </c>
       <c r="G726" s="3"/>
     </row>
     <row r="727" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A727" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B727">
         <v>2034</v>
@@ -15378,16 +15378,16 @@
         <v>8</v>
       </c>
       <c r="E727" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F727" s="3">
-        <v>1.0108711289835646</v>
+        <v>1.0178559493587218</v>
       </c>
       <c r="G727" s="3"/>
     </row>
     <row r="728" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A728" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B728">
         <v>2034</v>
@@ -15399,16 +15399,16 @@
         <v>8</v>
       </c>
       <c r="E728" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F728" s="3">
-        <v>1.0093086901096024</v>
+        <v>1.0108711289835646</v>
       </c>
       <c r="G728" s="3"/>
     </row>
     <row r="729" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A729" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B729">
         <v>2034</v>
@@ -15420,16 +15420,16 @@
         <v>8</v>
       </c>
       <c r="E729" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F729" s="3">
-        <v>1.0165936730302874</v>
+        <v>1.0093086901096024</v>
       </c>
       <c r="G729" s="3"/>
     </row>
     <row r="730" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A730" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B730">
         <v>2034</v>
@@ -15438,19 +15438,19 @@
         <v>17</v>
       </c>
       <c r="D730" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E730" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F730" s="3">
-        <v>1.0177161351629715</v>
+        <v>1.0165936730302874</v>
       </c>
       <c r="G730" s="3"/>
     </row>
     <row r="731" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A731" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B731">
         <v>2034</v>
@@ -15462,16 +15462,16 @@
         <v>12</v>
       </c>
       <c r="E731" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F731" s="3">
-        <v>1.0107728585851152</v>
+        <v>1.0177161351629715</v>
       </c>
       <c r="G731" s="3"/>
     </row>
     <row r="732" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A732" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B732">
         <v>2034</v>
@@ -15483,16 +15483,16 @@
         <v>12</v>
       </c>
       <c r="E732" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F732" s="3">
-        <v>1.0092410873187045</v>
+        <v>1.0107728585851152</v>
       </c>
       <c r="G732" s="3"/>
     </row>
     <row r="733" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A733" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B733">
         <v>2034</v>
@@ -15504,16 +15504,16 @@
         <v>12</v>
       </c>
       <c r="E733" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F733" s="3">
-        <v>1.0164877828214005</v>
+        <v>1.0092410873187045</v>
       </c>
       <c r="G733" s="3"/>
     </row>
     <row r="734" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A734" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B734">
         <v>2034</v>
@@ -15522,19 +15522,19 @@
         <v>17</v>
       </c>
       <c r="D734" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E734" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F734" s="3">
-        <v>1.0188089139105294</v>
+        <v>1.0164877828214005</v>
       </c>
       <c r="G734" s="3"/>
     </row>
     <row r="735" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A735" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B735">
         <v>2034</v>
@@ -15546,16 +15546,16 @@
         <v>13</v>
       </c>
       <c r="E735" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F735" s="3">
-        <v>1.0115473767392751</v>
+        <v>1.0188089139105294</v>
       </c>
       <c r="G735" s="3"/>
     </row>
     <row r="736" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A736" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B736">
         <v>2034</v>
@@ -15567,16 +15567,16 @@
         <v>13</v>
       </c>
       <c r="E736" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F736" s="3">
-        <v>1.0097704300620434</v>
+        <v>1.0115473767392751</v>
       </c>
       <c r="G736" s="3"/>
     </row>
     <row r="737" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A737" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B737">
         <v>2034</v>
@@ -15588,16 +15588,16 @@
         <v>13</v>
       </c>
       <c r="E737" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F737" s="3">
-        <v>1.0173102497537005</v>
+        <v>1.0097704300620434</v>
       </c>
       <c r="G737" s="3"/>
     </row>
     <row r="738" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A738" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B738">
         <v>2034</v>
@@ -15606,19 +15606,19 @@
         <v>17</v>
       </c>
       <c r="D738" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E738" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F738" s="3">
-        <v>1.0122088256573842</v>
+        <v>1.0173102497537005</v>
       </c>
       <c r="G738" s="3"/>
     </row>
     <row r="739" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A739" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B739">
         <v>2034</v>
@@ -15630,16 +15630,16 @@
         <v>14</v>
       </c>
       <c r="E739" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F739" s="3">
-        <v>1.0070838219177198</v>
+        <v>1.0122088256573842</v>
       </c>
       <c r="G739" s="3"/>
     </row>
     <row r="740" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A740" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B740">
         <v>2034</v>
@@ -15651,16 +15651,16 @@
         <v>14</v>
       </c>
       <c r="E740" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F740" s="3">
-        <v>1.0065055016002717</v>
+        <v>1.0070838219177198</v>
       </c>
       <c r="G740" s="3"/>
     </row>
     <row r="741" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A741" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B741">
         <v>2034</v>
@@ -15672,16 +15672,16 @@
         <v>14</v>
       </c>
       <c r="E741" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F741" s="3">
-        <v>1.0120452390150019</v>
+        <v>1.0065055016002717</v>
       </c>
       <c r="G741" s="3"/>
     </row>
     <row r="742" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A742" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B742">
         <v>2034</v>
@@ -15690,19 +15690,19 @@
         <v>17</v>
       </c>
       <c r="D742" t="s">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="E742" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F742" s="3">
-        <v>1.0180653873328906</v>
+        <v>1.0120452390150019</v>
       </c>
       <c r="G742" s="3"/>
     </row>
     <row r="743" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A743" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B743">
         <v>2034</v>
@@ -15714,16 +15714,16 @@
         <v>53</v>
       </c>
       <c r="E743" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F743" s="3">
-        <v>1.0110187850643273</v>
+        <v>1.0180653873328906</v>
       </c>
       <c r="G743" s="3"/>
     </row>
     <row r="744" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A744" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B744">
         <v>2034</v>
@@ -15735,16 +15735,16 @@
         <v>53</v>
       </c>
       <c r="E744" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F744" s="3">
-        <v>1.0094110041571775</v>
+        <v>1.0110187850643273</v>
       </c>
       <c r="G744" s="3"/>
     </row>
     <row r="745" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A745" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B745">
         <v>2034</v>
@@ -15756,37 +15756,37 @@
         <v>53</v>
       </c>
       <c r="E745" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F745" s="3">
-        <v>1.0167529044908412</v>
+        <v>1.0094110041571775</v>
       </c>
       <c r="G745" s="3"/>
     </row>
     <row r="746" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A746" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B746">
-        <v>2050</v>
+        <v>2034</v>
       </c>
       <c r="C746" t="s">
         <v>17</v>
       </c>
       <c r="D746" t="s">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="E746" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F746" s="3">
-        <v>1.0314408464477891</v>
+        <v>1.0167529044908412</v>
       </c>
       <c r="G746" s="3"/>
     </row>
     <row r="747" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A747" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B747">
         <v>2050</v>
@@ -15798,16 +15798,16 @@
         <v>8</v>
       </c>
       <c r="E747" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F747" s="3">
-        <v>1.0090625835218237</v>
+        <v>1.0314408464477891</v>
       </c>
       <c r="G747" s="3"/>
     </row>
     <row r="748" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A748" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B748">
         <v>2050</v>
@@ -15819,16 +15819,16 @@
         <v>8</v>
       </c>
       <c r="E748" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F748" s="3">
-        <v>1.0088217875674168</v>
+        <v>1.0090625835218237</v>
       </c>
       <c r="G748" s="3"/>
     </row>
     <row r="749" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A749" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B749">
         <v>2050</v>
@@ -15840,16 +15840,16 @@
         <v>8</v>
       </c>
       <c r="E749" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F749" s="3">
-        <v>1.0155763165435689</v>
+        <v>1.0088217875674168</v>
       </c>
       <c r="G749" s="3"/>
     </row>
     <row r="750" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A750" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B750">
         <v>2050</v>
@@ -15858,19 +15858,19 @@
         <v>17</v>
       </c>
       <c r="D750" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E750" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F750" s="3">
-        <v>1.0311883455840931</v>
+        <v>1.0155763165435689</v>
       </c>
       <c r="G750" s="3"/>
     </row>
     <row r="751" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A751" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B751">
         <v>2050</v>
@@ -15882,16 +15882,16 @@
         <v>12</v>
       </c>
       <c r="E751" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F751" s="3">
-        <v>1.0089790531368923</v>
+        <v>1.0311883455840931</v>
       </c>
       <c r="G751" s="3"/>
     </row>
     <row r="752" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A752" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B752">
         <v>2050</v>
@@ -15903,16 +15903,16 @@
         <v>12</v>
       </c>
       <c r="E752" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F752" s="3">
-        <v>1.0087474681575572</v>
+        <v>1.0089790531368923</v>
       </c>
       <c r="G752" s="3"/>
     </row>
     <row r="753" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A753" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B753">
         <v>2050</v>
@@ -15924,16 +15924,16 @@
         <v>12</v>
       </c>
       <c r="E753" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F753" s="3">
-        <v>1.0154404923593299</v>
+        <v>1.0087474681575572</v>
       </c>
       <c r="G753" s="3"/>
     </row>
     <row r="754" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A754" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B754">
         <v>2050</v>
@@ -15942,19 +15942,19 @@
         <v>17</v>
       </c>
       <c r="D754" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E754" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F754" s="3">
-        <v>1.0331646036143496</v>
+        <v>1.0154404923593299</v>
       </c>
       <c r="G754" s="3"/>
     </row>
     <row r="755" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A755" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B755">
         <v>2050</v>
@@ -15966,16 +15966,16 @@
         <v>13</v>
       </c>
       <c r="E755" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F755" s="3">
-        <v>1.0096382104321062</v>
+        <v>1.0331646036143496</v>
       </c>
       <c r="G755" s="3"/>
     </row>
     <row r="756" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A756" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B756">
         <v>2050</v>
@@ -15987,16 +15987,16 @@
         <v>13</v>
       </c>
       <c r="E756" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F756" s="3">
-        <v>1.0093328872234832</v>
+        <v>1.0096382104321062</v>
       </c>
       <c r="G756" s="3"/>
     </row>
     <row r="757" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A757" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B757">
         <v>2050</v>
@@ -16008,16 +16008,16 @@
         <v>13</v>
       </c>
       <c r="E757" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F757" s="3">
-        <v>1.0165125768888763</v>
+        <v>1.0093328872234832</v>
       </c>
       <c r="G757" s="3"/>
     </row>
     <row r="758" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A758" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B758">
         <v>2050</v>
@@ -16026,19 +16026,19 @@
         <v>17</v>
       </c>
       <c r="D758" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E758" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F758" s="3">
-        <v>1.0213229703232374</v>
+        <v>1.0165125768888763</v>
       </c>
       <c r="G758" s="3"/>
     </row>
     <row r="759" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A759" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B759">
         <v>2050</v>
@@ -16050,16 +16050,16 @@
         <v>14</v>
       </c>
       <c r="E759" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F759" s="3">
-        <v>1.0058648514021327</v>
+        <v>1.0213229703232374</v>
       </c>
       <c r="G759" s="3"/>
     </row>
     <row r="760" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A760" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B760">
         <v>2050</v>
@@ -16071,16 +16071,16 @@
         <v>14</v>
       </c>
       <c r="E760" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F760" s="3">
-        <v>1.0058829704467913</v>
+        <v>1.0058648514021327</v>
       </c>
       <c r="G760" s="3"/>
     </row>
     <row r="761" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A761" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B761">
         <v>2050</v>
@@ -16092,16 +16092,16 @@
         <v>14</v>
       </c>
       <c r="E761" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F761" s="3">
-        <v>1.0102664050263517</v>
+        <v>1.0058829704467913</v>
       </c>
       <c r="G761" s="3"/>
     </row>
     <row r="762" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A762" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B762">
         <v>2050</v>
@@ -16110,19 +16110,19 @@
         <v>17</v>
       </c>
       <c r="D762" t="s">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="E762" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F762" s="3">
-        <v>1.0318192774524944</v>
+        <v>1.0102664050263517</v>
       </c>
       <c r="G762" s="3"/>
     </row>
     <row r="763" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A763" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B763">
         <v>2050</v>
@@ -16134,16 +16134,16 @@
         <v>53</v>
       </c>
       <c r="E763" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F763" s="3">
-        <v>1.0091881482913909</v>
+        <v>1.0318192774524944</v>
       </c>
       <c r="G763" s="3"/>
     </row>
     <row r="764" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A764" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B764">
         <v>2050</v>
@@ -16155,16 +16155,16 @@
         <v>53</v>
       </c>
       <c r="E764" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F764" s="3">
-        <v>1.0089341249526491</v>
+        <v>1.0091881482913909</v>
       </c>
       <c r="G764" s="3"/>
     </row>
     <row r="765" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A765" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B765">
         <v>2050</v>
@@ -16176,37 +16176,37 @@
         <v>53</v>
       </c>
       <c r="E765" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F765" s="3">
-        <v>1.0157817716477346</v>
+        <v>1.0089341249526491</v>
       </c>
       <c r="G765" s="3"/>
     </row>
     <row r="766" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A766" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B766">
-        <v>2023</v>
+        <v>2050</v>
       </c>
       <c r="C766" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D766" t="s">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="E766" t="s">
-        <v>55</v>
+        <v>11</v>
       </c>
       <c r="F766" s="3">
-        <v>1.007903765988031</v>
+        <v>1.0157817716477346</v>
       </c>
       <c r="G766" s="3"/>
     </row>
     <row r="767" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A767" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B767">
         <v>2023</v>
@@ -16218,16 +16218,16 @@
         <v>8</v>
       </c>
       <c r="E767" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F767" s="3">
-        <v>1.0114839611671504</v>
+        <v>1.007903765988031</v>
       </c>
       <c r="G767" s="3"/>
     </row>
     <row r="768" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A768" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B768">
         <v>2023</v>
@@ -16239,16 +16239,16 @@
         <v>8</v>
       </c>
       <c r="E768" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F768" s="3">
-        <v>1.0439932102839258</v>
+        <v>1.0114839611671504</v>
       </c>
       <c r="G768" s="3"/>
     </row>
     <row r="769" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A769" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B769">
         <v>2023</v>
@@ -16260,16 +16260,16 @@
         <v>8</v>
       </c>
       <c r="E769" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F769" s="3">
-        <v>1.0539573026231246</v>
+        <v>1.0439932102839258</v>
       </c>
       <c r="G769" s="3"/>
     </row>
     <row r="770" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A770" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B770">
         <v>2023</v>
@@ -16281,16 +16281,16 @@
         <v>8</v>
       </c>
       <c r="E770" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F770" s="3">
-        <v>1.0335137230971052</v>
+        <v>1.0539573026231246</v>
       </c>
       <c r="G770" s="3"/>
     </row>
     <row r="771" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A771" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B771">
         <v>2023</v>
@@ -16299,19 +16299,19 @@
         <v>19</v>
       </c>
       <c r="D771" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E771" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F771" s="3">
-        <v>1.0073230543854415</v>
+        <v>1.0335137230971052</v>
       </c>
       <c r="G771" s="3"/>
     </row>
     <row r="772" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A772" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B772">
         <v>2023</v>
@@ -16323,16 +16323,16 @@
         <v>13</v>
       </c>
       <c r="E772" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F772" s="3">
-        <v>1.0109199502092687</v>
+        <v>1.0073230543854415</v>
       </c>
       <c r="G772" s="3"/>
     </row>
     <row r="773" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A773" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B773">
         <v>2023</v>
@@ -16344,16 +16344,16 @@
         <v>13</v>
       </c>
       <c r="E773" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F773" s="3">
-        <v>1.0429139451555589</v>
+        <v>1.0109199502092687</v>
       </c>
       <c r="G773" s="3"/>
     </row>
     <row r="774" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A774" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B774">
         <v>2023</v>
@@ -16365,16 +16365,16 @@
         <v>13</v>
       </c>
       <c r="E774" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F774" s="3">
-        <v>1.0525231917888074</v>
+        <v>1.0429139451555589</v>
       </c>
       <c r="G774" s="3"/>
     </row>
     <row r="775" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A775" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B775">
         <v>2023</v>
@@ -16386,16 +16386,16 @@
         <v>13</v>
       </c>
       <c r="E775" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F775" s="3">
-        <v>1.0330538911598923</v>
+        <v>1.0525231917888074</v>
       </c>
       <c r="G775" s="3"/>
     </row>
     <row r="776" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A776" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B776">
         <v>2023</v>
@@ -16404,19 +16404,19 @@
         <v>19</v>
       </c>
       <c r="D776" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E776" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F776" s="3">
-        <v>1.0079059866817959</v>
+        <v>1.0330538911598923</v>
       </c>
       <c r="G776" s="3"/>
     </row>
     <row r="777" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A777" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B777">
         <v>2023</v>
@@ -16428,16 +16428,16 @@
         <v>14</v>
       </c>
       <c r="E777" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F777" s="3">
-        <v>1.0114860625365856</v>
+        <v>1.0079059866817959</v>
       </c>
       <c r="G777" s="3"/>
     </row>
     <row r="778" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A778" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B778">
         <v>2023</v>
@@ -16449,16 +16449,16 @@
         <v>14</v>
       </c>
       <c r="E778" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F778" s="3">
-        <v>1.0439979226043763</v>
+        <v>1.0114860625365856</v>
       </c>
       <c r="G778" s="3"/>
     </row>
     <row r="779" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A779" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B779">
         <v>2023</v>
@@ -16470,16 +16470,16 @@
         <v>14</v>
       </c>
       <c r="E779" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F779" s="3">
-        <v>1.0539633661297994</v>
+        <v>1.0439979226043763</v>
       </c>
       <c r="G779" s="3"/>
     </row>
     <row r="780" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A780" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B780">
         <v>2023</v>
@@ -16491,16 +16491,16 @@
         <v>14</v>
       </c>
       <c r="E780" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F780" s="3">
-        <v>1.0335155081214094</v>
+        <v>1.0539633661297994</v>
       </c>
       <c r="G780" s="3"/>
     </row>
     <row r="781" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A781" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B781">
         <v>2023</v>
@@ -16509,19 +16509,19 @@
         <v>19</v>
       </c>
       <c r="D781" t="s">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="E781" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F781" s="3">
-        <v>1.0079098068194479</v>
+        <v>1.0335155081214094</v>
       </c>
       <c r="G781" s="3"/>
     </row>
     <row r="782" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A782" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B782">
         <v>2023</v>
@@ -16533,16 +16533,16 @@
         <v>53</v>
       </c>
       <c r="E782" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F782" s="3">
-        <v>1.0114896764440671</v>
+        <v>1.0079098068194479</v>
       </c>
       <c r="G782" s="3"/>
     </row>
     <row r="783" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A783" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B783">
         <v>2023</v>
@@ -16554,16 +16554,16 @@
         <v>53</v>
       </c>
       <c r="E783" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F783" s="3">
-        <v>1.0440038184559426</v>
+        <v>1.0114896764440671</v>
       </c>
       <c r="G783" s="3"/>
     </row>
     <row r="784" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A784" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B784">
         <v>2023</v>
@@ -16575,37 +16575,37 @@
         <v>53</v>
       </c>
       <c r="E784" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F784" s="3">
-        <v>1.0539714422948396</v>
+        <v>1.0440038184559426</v>
       </c>
       <c r="G784" s="3"/>
     </row>
     <row r="785" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A785" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B785">
-        <v>2034</v>
+        <v>2023</v>
       </c>
       <c r="C785" t="s">
         <v>19</v>
       </c>
       <c r="D785" t="s">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="E785" t="s">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="F785" s="3">
-        <v>1.0352053456525834</v>
+        <v>1.0539714422948396</v>
       </c>
       <c r="G785" s="3"/>
     </row>
     <row r="786" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A786" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B786">
         <v>2034</v>
@@ -16617,16 +16617,16 @@
         <v>8</v>
       </c>
       <c r="E786" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F786" s="3">
-        <v>1.0537744433707112</v>
+        <v>1.0352053456525834</v>
       </c>
       <c r="G786" s="3"/>
     </row>
     <row r="787" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A787" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B787">
         <v>2034</v>
@@ -16638,16 +16638,16 @@
         <v>8</v>
       </c>
       <c r="E787" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F787" s="3">
-        <v>1.0446814151892905</v>
+        <v>1.0537744433707112</v>
       </c>
       <c r="G787" s="3"/>
     </row>
     <row r="788" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A788" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B788">
         <v>2034</v>
@@ -16659,16 +16659,16 @@
         <v>8</v>
       </c>
       <c r="E788" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F788" s="3">
-        <v>1.0514683435102785</v>
+        <v>1.0446814151892905</v>
       </c>
       <c r="G788" s="3"/>
     </row>
     <row r="789" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A789" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B789">
         <v>2034</v>
@@ -16680,16 +16680,16 @@
         <v>8</v>
       </c>
       <c r="E789" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F789" s="3">
-        <v>1.0435164725581272</v>
+        <v>1.0514683435102785</v>
       </c>
       <c r="G789" s="3"/>
     </row>
     <row r="790" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A790" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B790">
         <v>2034</v>
@@ -16698,19 +16698,19 @@
         <v>19</v>
       </c>
       <c r="D790" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E790" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F790" s="3">
-        <v>1.0323682152528169</v>
+        <v>1.0435164725581272</v>
       </c>
       <c r="G790" s="3"/>
     </row>
     <row r="791" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A791" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B791">
         <v>2034</v>
@@ -16722,16 +16722,16 @@
         <v>13</v>
       </c>
       <c r="E791" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F791" s="3">
-        <v>1.0507298292781448</v>
+        <v>1.0323682152528169</v>
       </c>
       <c r="G791" s="3"/>
     </row>
     <row r="792" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A792" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B792">
         <v>2034</v>
@@ -16743,16 +16743,16 @@
         <v>13</v>
       </c>
       <c r="E792" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F792" s="3">
-        <v>1.0434295434974614</v>
+        <v>1.0507298292781448</v>
       </c>
       <c r="G792" s="3"/>
     </row>
     <row r="793" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A793" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B793">
         <v>2034</v>
@@ -16764,16 +16764,16 @@
         <v>13</v>
       </c>
       <c r="E793" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F793" s="3">
-        <v>1.0499987178350598</v>
+        <v>1.0434295434974614</v>
       </c>
       <c r="G793" s="3"/>
     </row>
     <row r="794" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A794" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B794">
         <v>2034</v>
@@ -16785,16 +16785,16 @@
         <v>13</v>
       </c>
       <c r="E794" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F794" s="3">
-        <v>1.0426511687919882</v>
+        <v>1.0499987178350598</v>
       </c>
       <c r="G794" s="3"/>
     </row>
     <row r="795" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A795" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B795">
         <v>2034</v>
@@ -16803,19 +16803,19 @@
         <v>19</v>
       </c>
       <c r="D795" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E795" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F795" s="3">
-        <v>1.0352162793830915</v>
+        <v>1.0426511687919882</v>
       </c>
       <c r="G795" s="3"/>
     </row>
     <row r="796" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A796" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B796">
         <v>2034</v>
@@ -16827,16 +16827,16 @@
         <v>14</v>
       </c>
       <c r="E796" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F796" s="3">
-        <v>1.0537858774568993</v>
+        <v>1.0352162793830915</v>
       </c>
       <c r="G796" s="3"/>
     </row>
     <row r="797" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A797" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B797">
         <v>2034</v>
@@ -16848,16 +16848,16 @@
         <v>14</v>
       </c>
       <c r="E797" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F797" s="3">
-        <v>1.0446868815084347</v>
+        <v>1.0537858774568993</v>
       </c>
       <c r="G797" s="3"/>
     </row>
     <row r="798" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A798" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B798">
         <v>2034</v>
@@ -16869,16 +16869,16 @@
         <v>14</v>
       </c>
       <c r="E798" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F798" s="3">
-        <v>1.0514745585176974</v>
+        <v>1.0446868815084347</v>
       </c>
       <c r="G798" s="3"/>
     </row>
     <row r="799" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A799" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B799">
         <v>2034</v>
@@ -16890,16 +16890,16 @@
         <v>14</v>
       </c>
       <c r="E799" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F799" s="3">
-        <v>1.0435198527928728</v>
+        <v>1.0514745585176974</v>
       </c>
       <c r="G799" s="3"/>
     </row>
     <row r="800" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A800" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B800">
         <v>2034</v>
@@ -16908,19 +16908,19 @@
         <v>19</v>
       </c>
       <c r="D800" t="s">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="E800" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F800" s="3">
-        <v>1.0352350895941367</v>
+        <v>1.0435198527928728</v>
       </c>
       <c r="G800" s="3"/>
     </row>
     <row r="801" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A801" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B801">
         <v>2034</v>
@@ -16932,16 +16932,16 @@
         <v>53</v>
       </c>
       <c r="E801" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F801" s="3">
-        <v>1.0538055432331599</v>
+        <v>1.0352350895941367</v>
       </c>
       <c r="G801" s="3"/>
     </row>
     <row r="802" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A802" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B802">
         <v>2034</v>
@@ -16953,16 +16953,16 @@
         <v>53</v>
       </c>
       <c r="E802" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F802" s="3">
-        <v>1.044693765748254</v>
+        <v>1.0538055432331599</v>
       </c>
       <c r="G802" s="3"/>
     </row>
     <row r="803" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A803" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B803">
         <v>2034</v>
@@ -16974,16 +16974,16 @@
         <v>53</v>
       </c>
       <c r="E803" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F803" s="3">
-        <v>1.0514828638297036</v>
+        <v>1.044693765748254</v>
       </c>
       <c r="G803" s="3"/>
     </row>
     <row r="804" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A804" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B804">
         <v>2034</v>
@@ -16995,37 +16995,37 @@
         <v>53</v>
       </c>
       <c r="E804" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F804" s="3">
-        <v>1.043524961306231</v>
+        <v>1.0514828638297036</v>
       </c>
       <c r="G804" s="3"/>
     </row>
     <row r="805" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A805" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B805">
-        <v>2050</v>
+        <v>2034</v>
       </c>
       <c r="C805" t="s">
         <v>19</v>
       </c>
       <c r="D805" t="s">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="E805" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F805" s="3">
-        <v>1.0606805579244005</v>
+        <v>1.043524961306231</v>
       </c>
       <c r="G805" s="3"/>
     </row>
     <row r="806" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A806" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B806">
         <v>2050</v>
@@ -17037,16 +17037,16 @@
         <v>8</v>
       </c>
       <c r="E806" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F806" s="3">
-        <v>1.0974091022051089</v>
+        <v>1.0606805579244005</v>
       </c>
       <c r="G806" s="3"/>
     </row>
     <row r="807" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A807" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B807">
         <v>2050</v>
@@ -17058,16 +17058,16 @@
         <v>8</v>
       </c>
       <c r="E807" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F807" s="3">
-        <v>1.0448589580191896</v>
+        <v>1.0974091022051089</v>
       </c>
       <c r="G807" s="3"/>
     </row>
     <row r="808" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A808" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B808">
         <v>2050</v>
@@ -17079,16 +17079,16 @@
         <v>8</v>
       </c>
       <c r="E808" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F808" s="3">
-        <v>1.049824967209223</v>
+        <v>1.0448589580191896</v>
       </c>
       <c r="G808" s="3"/>
     </row>
     <row r="809" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A809" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B809">
         <v>2050</v>
@@ -17100,16 +17100,16 @@
         <v>8</v>
       </c>
       <c r="E809" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F809" s="3">
-        <v>1.0489694523611228</v>
+        <v>1.049824967209223</v>
       </c>
       <c r="G809" s="3"/>
     </row>
     <row r="810" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A810" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B810">
         <v>2050</v>
@@ -17118,19 +17118,19 @@
         <v>19</v>
       </c>
       <c r="D810" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E810" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F810" s="3">
-        <v>1.0554636719122097</v>
+        <v>1.0489694523611228</v>
       </c>
       <c r="G810" s="3"/>
     </row>
     <row r="811" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A811" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B811">
         <v>2050</v>
@@ -17142,16 +17142,16 @@
         <v>13</v>
       </c>
       <c r="E811" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F811" s="3">
-        <v>1.0912339165171296</v>
+        <v>1.0554636719122097</v>
       </c>
       <c r="G811" s="3"/>
     </row>
     <row r="812" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A812" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B812">
         <v>2050</v>
@@ -17163,16 +17163,16 @@
         <v>13</v>
       </c>
       <c r="E812" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F812" s="3">
-        <v>1.0430166398023553</v>
+        <v>1.0912339165171296</v>
       </c>
       <c r="G812" s="3"/>
     </row>
     <row r="813" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A813" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B813">
         <v>2050</v>
@@ -17184,16 +17184,16 @@
         <v>13</v>
       </c>
       <c r="E813" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F813" s="3">
-        <v>1.0478107792235023</v>
+        <v>1.0430166398023553</v>
       </c>
       <c r="G813" s="3"/>
     </row>
     <row r="814" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A814" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B814">
         <v>2050</v>
@@ -17205,16 +17205,16 @@
         <v>13</v>
       </c>
       <c r="E814" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F814" s="3">
-        <v>1.047436293772313</v>
+        <v>1.0478107792235023</v>
       </c>
       <c r="G814" s="3"/>
     </row>
     <row r="815" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A815" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B815">
         <v>2050</v>
@@ -17223,19 +17223,19 @@
         <v>19</v>
       </c>
       <c r="D815" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E815" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F815" s="3">
-        <v>1.060700781659313</v>
+        <v>1.047436293772313</v>
       </c>
       <c r="G815" s="3"/>
     </row>
     <row r="816" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A816" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B816">
         <v>2050</v>
@@ -17247,16 +17247,16 @@
         <v>14</v>
       </c>
       <c r="E816" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F816" s="3">
-        <v>1.0974324616075366</v>
+        <v>1.060700781659313</v>
       </c>
       <c r="G816" s="3"/>
     </row>
     <row r="817" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A817" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B817">
         <v>2050</v>
@@ -17268,16 +17268,16 @@
         <v>14</v>
       </c>
       <c r="E817" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F817" s="3">
-        <v>1.0448668704369459</v>
+        <v>1.0974324616075366</v>
       </c>
       <c r="G817" s="3"/>
     </row>
     <row r="818" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A818" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B818">
         <v>2050</v>
@@ -17289,16 +17289,16 @@
         <v>14</v>
       </c>
       <c r="E818" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F818" s="3">
-        <v>1.049833458793004</v>
+        <v>1.0448668704369459</v>
       </c>
       <c r="G818" s="3"/>
     </row>
     <row r="819" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A819" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B819">
         <v>2050</v>
@@ -17310,16 +17310,16 @@
         <v>14</v>
       </c>
       <c r="E819" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F819" s="3">
-        <v>1.0489755124236584</v>
+        <v>1.049833458793004</v>
       </c>
       <c r="G819" s="3"/>
     </row>
     <row r="820" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A820" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B820">
         <v>2050</v>
@@ -17328,19 +17328,19 @@
         <v>19</v>
       </c>
       <c r="D820" t="s">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="E820" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F820" s="3">
-        <v>1.06073557639098</v>
+        <v>1.0489755124236584</v>
       </c>
       <c r="G820" s="3"/>
     </row>
     <row r="821" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A821" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B821">
         <v>2050</v>
@@ -17352,16 +17352,16 @@
         <v>53</v>
       </c>
       <c r="E821" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F821" s="3">
-        <v>1.0974726410084363</v>
+        <v>1.06073557639098</v>
       </c>
       <c r="G821" s="3"/>
     </row>
     <row r="822" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A822" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B822">
         <v>2050</v>
@@ -17373,16 +17373,16 @@
         <v>53</v>
       </c>
       <c r="E822" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="F822" s="3">
-        <v>1.0448773993507929</v>
+        <v>1.0974726410084363</v>
       </c>
       <c r="G822" s="3"/>
     </row>
     <row r="823" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A823" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B823">
         <v>2050</v>
@@ -17394,16 +17394,16 @@
         <v>53</v>
       </c>
       <c r="E823" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F823" s="3">
-        <v>1.0498451251267131</v>
+        <v>1.0448773993507929</v>
       </c>
       <c r="G823" s="3"/>
     </row>
     <row r="824" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A824" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="B824">
         <v>2050</v>
@@ -17415,12 +17415,53 @@
         <v>53</v>
       </c>
       <c r="E824" t="s">
+        <v>20</v>
+      </c>
+      <c r="F824" s="3">
+        <v>1.0498451251267131</v>
+      </c>
+      <c r="G824" s="3"/>
+    </row>
+    <row r="825" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A825" t="s">
+        <v>69</v>
+      </c>
+      <c r="B825">
+        <v>2050</v>
+      </c>
+      <c r="C825" t="s">
+        <v>19</v>
+      </c>
+      <c r="D825" t="s">
+        <v>53</v>
+      </c>
+      <c r="E825" t="s">
         <v>21</v>
       </c>
-      <c r="F824" s="3">
+      <c r="F825" s="3">
         <v>1.0489846719923754</v>
       </c>
-      <c r="G824" s="3"/>
+      <c r="G825" s="3"/>
+    </row>
+    <row r="826" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A826" t="s">
+        <v>69</v>
+      </c>
+      <c r="B826">
+        <v>2023</v>
+      </c>
+      <c r="C826" t="s">
+        <v>19</v>
+      </c>
+      <c r="D826" t="s">
+        <v>53</v>
+      </c>
+      <c r="E826" t="s">
+        <v>21</v>
+      </c>
+      <c r="F826" s="3">
+        <v>1.0539714422948396</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -17751,7 +17792,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{684F6E1A-D3EC-47A8-91AD-3E7ADA2F1FE3}">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
@@ -17800,11 +17841,11 @@
         <v>1</v>
       </c>
       <c r="B3" t="str">
-        <f t="shared" ref="B3:B25" si="0">_xlfn.CONCAT(D3:E3)</f>
+        <f t="shared" ref="B3:B16" si="0">_xlfn.CONCAT(D3:E3)</f>
         <v>EO</v>
       </c>
       <c r="C3" s="2">
-        <f t="shared" ref="C3:C26" si="1">1/25</f>
+        <f t="shared" ref="C3:C17" si="1">1/25</f>
         <v>0.04</v>
       </c>
       <c r="D3" t="s">
@@ -17816,11 +17857,11 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
-        <v>EB</v>
+        <v>EP</v>
       </c>
       <c r="C4" s="2">
         <f t="shared" si="1"/>
@@ -17830,16 +17871,16 @@
         <v>68</v>
       </c>
       <c r="E4" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
-        <v>EP</v>
+        <v>EN</v>
       </c>
       <c r="C5" s="2">
         <f t="shared" si="1"/>
@@ -17849,35 +17890,35 @@
         <v>68</v>
       </c>
       <c r="E5" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
-        <v>EN</v>
+        <v>OE</v>
       </c>
       <c r="C6" s="2">
         <f t="shared" si="1"/>
         <v>0.04</v>
       </c>
       <c r="D6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" t="s">
         <v>68</v>
-      </c>
-      <c r="E6" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
-        <v>OE</v>
+        <v>OO</v>
       </c>
       <c r="C7" s="2">
         <f t="shared" si="1"/>
@@ -17887,16 +17928,16 @@
         <v>15</v>
       </c>
       <c r="E7" t="s">
-        <v>68</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
-        <v>OO</v>
+        <v>OP</v>
       </c>
       <c r="C8" s="2">
         <f t="shared" si="1"/>
@@ -17906,16 +17947,16 @@
         <v>15</v>
       </c>
       <c r="E8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
-        <v>OB</v>
+        <v>ON</v>
       </c>
       <c r="C9" s="2">
         <f t="shared" si="1"/>
@@ -17925,334 +17966,163 @@
         <v>15</v>
       </c>
       <c r="E9" t="s">
-        <v>6</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
-        <v>OP</v>
+        <v>PE</v>
       </c>
       <c r="C10" s="2">
         <f t="shared" si="1"/>
         <v>0.04</v>
       </c>
       <c r="D10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E10" t="s">
-        <v>16</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
-        <v>ON</v>
+        <v>PO</v>
       </c>
       <c r="C11" s="2">
         <f t="shared" si="1"/>
         <v>0.04</v>
       </c>
       <c r="D11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E11" t="s">
-        <v>69</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
-        <v>BE</v>
+        <v>PP</v>
       </c>
       <c r="C12" s="2">
         <f t="shared" si="1"/>
         <v>0.04</v>
       </c>
       <c r="D12" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="E12" t="s">
-        <v>68</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
-        <v>BO</v>
+        <v>PN</v>
       </c>
       <c r="C13" s="2">
         <f t="shared" si="1"/>
         <v>0.04</v>
       </c>
       <c r="D13" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="E13" t="s">
-        <v>15</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
-        <v>BB</v>
+        <v>NE</v>
       </c>
       <c r="C14" s="2">
         <f t="shared" si="1"/>
         <v>0.04</v>
       </c>
       <c r="D14" t="s">
-        <v>6</v>
+        <v>69</v>
       </c>
       <c r="E14" t="s">
-        <v>6</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
-        <v>BP</v>
+        <v>NO</v>
       </c>
       <c r="C15" s="2">
         <f t="shared" si="1"/>
         <v>0.04</v>
       </c>
       <c r="D15" t="s">
-        <v>6</v>
+        <v>69</v>
       </c>
       <c r="E15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
-        <v>BN</v>
+        <v>NP</v>
       </c>
       <c r="C16" s="2">
         <f t="shared" si="1"/>
         <v>0.04</v>
       </c>
       <c r="D16" t="s">
-        <v>6</v>
+        <v>69</v>
       </c>
       <c r="E16" t="s">
-        <v>69</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="B17" t="str">
-        <f t="shared" si="0"/>
-        <v>PE</v>
+        <f t="shared" ref="B17" si="2">_xlfn.CONCAT(D17:E17)</f>
+        <v>NN</v>
       </c>
       <c r="C17" s="2">
         <f t="shared" si="1"/>
         <v>0.04</v>
       </c>
       <c r="D17" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="E17" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>16</v>
-      </c>
-      <c r="B18" t="str">
-        <f t="shared" si="0"/>
-        <v>PO</v>
-      </c>
-      <c r="C18" s="2">
-        <f t="shared" si="1"/>
-        <v>0.04</v>
-      </c>
-      <c r="D18" t="s">
-        <v>16</v>
-      </c>
-      <c r="E18" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>17</v>
-      </c>
-      <c r="B19" t="str">
-        <f t="shared" si="0"/>
-        <v>PB</v>
-      </c>
-      <c r="C19" s="2">
-        <f t="shared" si="1"/>
-        <v>0.04</v>
-      </c>
-      <c r="D19" t="s">
-        <v>16</v>
-      </c>
-      <c r="E19" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>18</v>
-      </c>
-      <c r="B20" t="str">
-        <f t="shared" si="0"/>
-        <v>PP</v>
-      </c>
-      <c r="C20" s="2">
-        <f t="shared" si="1"/>
-        <v>0.04</v>
-      </c>
-      <c r="D20" t="s">
-        <v>16</v>
-      </c>
-      <c r="E20" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>19</v>
-      </c>
-      <c r="B21" t="str">
-        <f t="shared" si="0"/>
-        <v>PN</v>
-      </c>
-      <c r="C21" s="2">
-        <f t="shared" si="1"/>
-        <v>0.04</v>
-      </c>
-      <c r="D21" t="s">
-        <v>16</v>
-      </c>
-      <c r="E21" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>20</v>
-      </c>
-      <c r="B22" t="str">
-        <f t="shared" si="0"/>
-        <v>NE</v>
-      </c>
-      <c r="C22" s="2">
-        <f t="shared" si="1"/>
-        <v>0.04</v>
-      </c>
-      <c r="D22" t="s">
-        <v>69</v>
-      </c>
-      <c r="E22" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>21</v>
-      </c>
-      <c r="B23" t="str">
-        <f t="shared" si="0"/>
-        <v>NO</v>
-      </c>
-      <c r="C23" s="2">
-        <f t="shared" si="1"/>
-        <v>0.04</v>
-      </c>
-      <c r="D23" t="s">
-        <v>69</v>
-      </c>
-      <c r="E23" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>22</v>
-      </c>
-      <c r="B24" t="str">
-        <f t="shared" si="0"/>
-        <v>NB</v>
-      </c>
-      <c r="C24" s="2">
-        <f t="shared" si="1"/>
-        <v>0.04</v>
-      </c>
-      <c r="D24" t="s">
-        <v>69</v>
-      </c>
-      <c r="E24" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <v>23</v>
-      </c>
-      <c r="B25" t="str">
-        <f t="shared" si="0"/>
-        <v>NP</v>
-      </c>
-      <c r="C25" s="2">
-        <f t="shared" si="1"/>
-        <v>0.04</v>
-      </c>
-      <c r="D25" t="s">
-        <v>69</v>
-      </c>
-      <c r="E25" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>24</v>
-      </c>
-      <c r="B26" t="str">
-        <f t="shared" ref="B26" si="2">_xlfn.CONCAT(D26:E26)</f>
-        <v>NN</v>
-      </c>
-      <c r="C26" s="2">
-        <f t="shared" si="1"/>
-        <v>0.04</v>
-      </c>
-      <c r="D26" t="s">
-        <v>69</v>
-      </c>
-      <c r="E26" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C27" s="2"/>
+      <c r="C18" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>